<commit_message>
feat: complete database wrapping, brand sanitization, and team revisions
- Database: package complete self-contained dump (database/mitra_kinerja_dump.sql) alongside updated schema.sql and seed_data.sql
- Brand: sanitize entity nomenclature to 'Kanwil Kementerian Hukum Kepri' across all UI, certificates, scripts, and database
- Manajemen Naskah: add PDF scan upload, annual work plan form, and Bidang reclassification
- Gate 0: add partnership type template dropdown and vertical downward form layout generator
- Baseline FIX: implement 7th Action column with single/multi PDF uploads, interactive PIC modals, Pelaksanaan count, and Eviden shortcut
- Penilaian: rename validation menu to 'Penilaian' and grant examiner direct access with visible monev milestones
- Alerts: add Pengampu and PIC role-tailored deadline warnings on Dashboard and Scorecard
</commit_message>
<xml_diff>
--- a/public/templates/template_gate0_dalam_negeri.xlsx
+++ b/public/templates/template_gate0_dalam_negeri.xlsx
@@ -172,13 +172,13 @@
     <t>Q1</t>
   </si>
   <si>
-    <t>K1.1: Kesesuaian dengan tugas pokok dan fungsi (Tusi) Kementerian Hukum dan HAM</t>
+    <t>K1.1: Kesesuaian dengan tugas pokok dan fungsi (Tusi) Kementerian Hukum</t>
   </si>
   <si>
     <t>YA</t>
   </si>
   <si>
-    <t>Sesuai Renstra Kanwil Kemenkumham Kepri</t>
+    <t>Sesuai Renstra Kanwil Kementerian Hukum Kepri</t>
   </si>
   <si>
     <t>Q2</t>
@@ -400,7 +400,7 @@
     <t>Pemicu 7: Publikasi, Penggunaan Logo, dan Branding Resmi</t>
   </si>
   <si>
-    <t>Sesuai pedoman humas Kemenkumham</t>
+    <t>Sesuai pedoman humas Kementerian Hukum</t>
   </si>
   <si>
     <t>BAGIAN IV: CATATAN &amp; HASIL REVIU VERIFIKATOR</t>

</xml_diff>

<commit_message>
feat: implement team revisions v2.2.1 and core hardenings
- Gate 0: embed native Excel data validation (YA/TIDAK) in C16:C33 and C35:C41, and enhance OpenXML coordinate parsing
- Manajemen Naskah: add evaluasi_per_tahun field with dynamic scorecard duration calculation (36 months / 4 = 9 cycles)
- Scorecard: add 7th progress card for Kegiatan Terkait and fix badge text wrapping
- Tindak Lanjut: add evidence file upload (PDF/Images/Docs up to 25MB) with download button in ledger
- UI/UX: add searchable combobox dropdown widget with autocomplete and keyboard navigation, plus instant search on portofolio.php
- Hardening: secure upload directories, date formatting (formatTanggalPanjang), and self-healing validation records
- Database: sync complete dump, schema, and seed data across all 13 tables
</commit_message>
<xml_diff>
--- a/public/templates/template_gate0_dalam_negeri.xlsx
+++ b/public/templates/template_gate0_dalam_negeri.xlsx
@@ -1160,5 +1160,13 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C16:C33">
+      <formula1>"YA,TIDAK"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C35:C41">
+      <formula1>"YA,TIDAK"</formula1>
+    </dataValidation>
+  </dataValidations>
 </worksheet>
 </file>
</xml_diff>